<commit_message>
Add mask UI and expand card configs
Introduce mask switching UI and extend card data for new mechanics. Added SwitchMaskButton prefab and runtime script; integrated MaskPanel and related UI elements into GamePlayPanel prefab. Overhauled cardtable.json: added types, names, localized descriptions, value arrays and mask mappings for many cards. Added generated enums (CardTypeEnum, MaskEnum) and updated CardConfig.cs, CardEnum.cs and GameLevelEnum.cs to reflect the new data. Updated source spreadsheets and .gitignore to ignore temporary .~*.xlsx files. These changes implement mask-related gameplay features and expand the card dataset.
</commit_message>
<xml_diff>
--- a/Configs/source/Datas/__enums__.xlsx
+++ b/Configs/source/Datas/__enums__.xlsx
@@ -1,10 +1,10 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="25600" windowHeight="12080" firstSheet="2"/>
+    <workbookView windowWidth="29100" windowHeight="12700" firstSheet="2" activeTab="6"/>
   </bookViews>
   <sheets>
     <sheet name="Card" sheetId="1" r:id="rId1"/>
@@ -13,6 +13,7 @@
     <sheet name="Intent" sheetId="5" r:id="rId4"/>
     <sheet name="GameMap" sheetId="3" r:id="rId5"/>
     <sheet name="GameLevel" sheetId="6" r:id="rId6"/>
+    <sheet name="Mask" sheetId="8" r:id="rId7"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -32,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="194" uniqueCount="80">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="223" uniqueCount="87">
   <si>
     <t>##var</t>
   </si>
@@ -272,6 +273,27 @@
   </si>
   <si>
     <t>第九关</t>
+  </si>
+  <si>
+    <t>MaskEnum</t>
+  </si>
+  <si>
+    <t>本我</t>
+  </si>
+  <si>
+    <t>阎王</t>
+  </si>
+  <si>
+    <t>十殿阎罗</t>
+  </si>
+  <si>
+    <t>黑白无常</t>
+  </si>
+  <si>
+    <t>孟婆</t>
+  </si>
+  <si>
+    <t>二郎神</t>
   </si>
 </sst>
 </file>
@@ -945,10 +967,10 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1">
       <alignment vertical="center"/>
@@ -1279,7 +1301,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:L37"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="16.8"/>
   <cols>
     <col min="2" max="2" width="19" customWidth="1"/>
     <col min="3" max="3" width="20.875" customWidth="1"/>
@@ -1314,13 +1336,13 @@
       <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="H1" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="2"/>
-      <c r="J1" s="2"/>
-      <c r="K1" s="2"/>
-      <c r="L1" s="2"/>
+      <c r="I1" s="3"/>
+      <c r="J1" s="3"/>
+      <c r="K1" s="3"/>
+      <c r="L1" s="3"/>
     </row>
     <row r="2" spans="1:12">
       <c r="A2" s="1" t="s">
@@ -1355,7 +1377,7 @@
       <c r="B3" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="C3" s="2" t="s">
         <v>13</v>
       </c>
       <c r="D3" s="1" t="s">
@@ -1378,7 +1400,7 @@
       </c>
       <c r="L3" s="1"/>
     </row>
-    <row r="4" spans="1:12">
+    <row r="4" spans="2:8">
       <c r="B4" t="s">
         <v>19</v>
       </c>
@@ -1389,62 +1411,62 @@
         <v>20</v>
       </c>
     </row>
-    <row r="5" spans="1:12">
+    <row r="5" spans="8:8">
       <c r="H5" s="5" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="6" spans="1:12">
+    <row r="6" spans="8:8">
       <c r="H6" s="5" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="7" spans="1:12">
+    <row r="7" spans="8:8">
       <c r="H7" s="5" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="8" spans="1:12">
+    <row r="8" spans="8:8">
       <c r="H8" s="5" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="9" spans="1:12">
+    <row r="9" spans="8:8">
       <c r="H9" s="5" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="10" spans="1:12">
+    <row r="10" spans="8:8">
       <c r="H10" s="5" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="11" spans="1:12">
+    <row r="11" spans="8:8">
       <c r="H11" s="5" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="12" spans="1:12">
+    <row r="12" spans="8:8">
       <c r="H12" s="5" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="13" spans="1:12">
+    <row r="13" spans="8:8">
       <c r="H13" s="5" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="14" spans="1:12">
+    <row r="14" spans="8:8">
       <c r="H14" s="5" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="15" spans="1:12">
+    <row r="15" spans="8:8">
       <c r="H15" s="5" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="16" spans="1:12">
+    <row r="16" spans="8:8">
       <c r="H16" s="4" t="s">
         <v>32</v>
       </c>
@@ -1568,7 +1590,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:L22"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="16.8"/>
   <cols>
     <col min="2" max="2" width="19" customWidth="1"/>
     <col min="3" max="3" width="20.875" customWidth="1"/>
@@ -1603,13 +1625,13 @@
       <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="H1" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="2"/>
-      <c r="J1" s="2"/>
-      <c r="K1" s="2"/>
-      <c r="L1" s="2"/>
+      <c r="I1" s="3"/>
+      <c r="J1" s="3"/>
+      <c r="K1" s="3"/>
+      <c r="L1" s="3"/>
     </row>
     <row r="2" spans="1:12">
       <c r="A2" s="1" t="s">
@@ -1644,7 +1666,7 @@
       <c r="B3" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="C3" s="2" t="s">
         <v>13</v>
       </c>
       <c r="D3" s="1" t="s">
@@ -1667,7 +1689,7 @@
       </c>
       <c r="L3" s="1"/>
     </row>
-    <row r="4" customFormat="1" spans="1:12">
+    <row r="4" customFormat="1" spans="2:8">
       <c r="B4" t="s">
         <v>54</v>
       </c>
@@ -1678,46 +1700,46 @@
         <v>55</v>
       </c>
     </row>
-    <row r="5" customFormat="1" spans="1:12">
+    <row r="5" customFormat="1" spans="8:8">
       <c r="H5" s="5" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="6" customFormat="1" spans="1:12">
+    <row r="6" customFormat="1" spans="8:8">
       <c r="H6" s="5" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="7" customFormat="1" spans="1:12">
+    <row r="7" customFormat="1" spans="8:8">
       <c r="H7" s="5" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="8" customFormat="1" spans="1:12">
+    <row r="8" customFormat="1" spans="8:8">
       <c r="H8" s="5"/>
     </row>
-    <row r="9" customFormat="1" spans="1:12">
+    <row r="9" customFormat="1" spans="8:8">
       <c r="H9" s="5"/>
     </row>
-    <row r="10" customFormat="1" spans="1:12">
+    <row r="10" customFormat="1" spans="8:8">
       <c r="H10" s="5"/>
     </row>
-    <row r="11" customFormat="1" spans="1:12">
+    <row r="11" customFormat="1" spans="8:8">
       <c r="H11" s="5"/>
     </row>
-    <row r="12" customFormat="1" spans="1:12">
+    <row r="12" customFormat="1" spans="8:8">
       <c r="H12" s="5"/>
     </row>
-    <row r="13" customFormat="1" spans="1:12">
+    <row r="13" customFormat="1" spans="8:8">
       <c r="H13" s="5"/>
     </row>
-    <row r="14" customFormat="1" spans="1:12">
+    <row r="14" customFormat="1" spans="8:8">
       <c r="H14" s="5"/>
     </row>
-    <row r="15" customFormat="1" spans="1:12">
+    <row r="15" customFormat="1" spans="8:8">
       <c r="H15" s="5"/>
     </row>
-    <row r="16" customFormat="1" spans="1:12">
+    <row r="16" customFormat="1" spans="8:8">
       <c r="H16" s="4"/>
     </row>
     <row r="17" customFormat="1" spans="8:8">
@@ -1751,7 +1773,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:L7"/>
-  <sheetFormatPr defaultColWidth="9.14166666666667" defaultRowHeight="14" outlineLevelRow="6"/>
+  <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="16.8" outlineLevelRow="6"/>
   <sheetData>
     <row r="1" spans="1:12">
       <c r="A1" s="1" t="s">
@@ -1775,13 +1797,13 @@
       <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="H1" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="2"/>
-      <c r="J1" s="2"/>
-      <c r="K1" s="2"/>
-      <c r="L1" s="2"/>
+      <c r="I1" s="3"/>
+      <c r="J1" s="3"/>
+      <c r="K1" s="3"/>
+      <c r="L1" s="3"/>
     </row>
     <row r="2" spans="1:12">
       <c r="A2" s="1" t="s">
@@ -1809,14 +1831,14 @@
         <v>6</v>
       </c>
     </row>
-    <row r="3" ht="168" spans="1:12">
+    <row r="3" ht="219" spans="1:12">
       <c r="A3" s="1" t="s">
         <v>11</v>
       </c>
       <c r="B3" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="C3" s="2" t="s">
         <v>13</v>
       </c>
       <c r="D3" s="1" t="s">
@@ -1839,7 +1861,7 @@
       </c>
       <c r="L3" s="1"/>
     </row>
-    <row r="4" spans="1:12">
+    <row r="4" spans="2:8">
       <c r="B4" t="s">
         <v>59</v>
       </c>
@@ -1850,15 +1872,15 @@
         <v>60</v>
       </c>
     </row>
-    <row r="5" spans="1:12">
+    <row r="5" spans="8:8">
       <c r="H5" s="4" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="6" spans="1:12">
+    <row r="6" spans="8:8">
       <c r="H6" s="4"/>
     </row>
-    <row r="7" spans="1:12">
+    <row r="7" spans="8:8">
       <c r="H7" s="4"/>
     </row>
   </sheetData>
@@ -1874,7 +1896,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:L7"/>
-  <sheetFormatPr defaultColWidth="9.14166666666667" defaultRowHeight="14" outlineLevelRow="6"/>
+  <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="16.8" outlineLevelRow="6"/>
   <sheetData>
     <row r="1" spans="1:12">
       <c r="A1" s="1" t="s">
@@ -1898,13 +1920,13 @@
       <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="H1" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="2"/>
-      <c r="J1" s="2"/>
-      <c r="K1" s="2"/>
-      <c r="L1" s="2"/>
+      <c r="I1" s="3"/>
+      <c r="J1" s="3"/>
+      <c r="K1" s="3"/>
+      <c r="L1" s="3"/>
     </row>
     <row r="2" spans="1:12">
       <c r="A2" s="1" t="s">
@@ -1932,14 +1954,14 @@
         <v>6</v>
       </c>
     </row>
-    <row r="3" ht="168" spans="1:12">
+    <row r="3" ht="219" spans="1:12">
       <c r="A3" s="1" t="s">
         <v>11</v>
       </c>
       <c r="B3" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="C3" s="2" t="s">
         <v>13</v>
       </c>
       <c r="D3" s="1" t="s">
@@ -1962,7 +1984,7 @@
       </c>
       <c r="L3" s="1"/>
     </row>
-    <row r="4" spans="1:12">
+    <row r="4" spans="2:8">
       <c r="B4" t="s">
         <v>62</v>
       </c>
@@ -1973,17 +1995,17 @@
         <v>55</v>
       </c>
     </row>
-    <row r="5" spans="1:12">
+    <row r="5" spans="8:8">
       <c r="H5" s="4" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="6" spans="1:12">
+    <row r="6" spans="8:8">
       <c r="H6" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="7" spans="1:12">
+    <row r="7" spans="8:8">
       <c r="H7" t="s">
         <v>65</v>
       </c>
@@ -2001,11 +2023,11 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:L23"/>
-  <sheetFormatPr defaultColWidth="9.14166666666667" defaultRowHeight="14"/>
+  <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="16.8"/>
   <cols>
     <col min="2" max="2" width="14.875" customWidth="1"/>
-    <col min="10" max="10" width="12.2" customWidth="1"/>
-    <col min="11" max="11" width="16.075" customWidth="1"/>
+    <col min="10" max="10" width="12.1964285714286" customWidth="1"/>
+    <col min="11" max="11" width="16.0714285714286" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:12">
@@ -2030,13 +2052,13 @@
       <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="H1" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="2"/>
-      <c r="J1" s="2"/>
-      <c r="K1" s="2"/>
-      <c r="L1" s="2"/>
+      <c r="I1" s="3"/>
+      <c r="J1" s="3"/>
+      <c r="K1" s="3"/>
+      <c r="L1" s="3"/>
     </row>
     <row r="2" spans="1:12">
       <c r="A2" s="1" t="s">
@@ -2064,14 +2086,14 @@
         <v>6</v>
       </c>
     </row>
-    <row r="3" ht="168" spans="1:12">
+    <row r="3" ht="219" spans="1:12">
       <c r="A3" s="1" t="s">
         <v>11</v>
       </c>
       <c r="B3" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="C3" s="2" t="s">
         <v>13</v>
       </c>
       <c r="D3" s="1" t="s">
@@ -2094,7 +2116,7 @@
       </c>
       <c r="L3" s="1"/>
     </row>
-    <row r="4" spans="1:12">
+    <row r="4" spans="2:11">
       <c r="B4" t="s">
         <v>66</v>
       </c>
@@ -2111,42 +2133,42 @@
         <v>68</v>
       </c>
     </row>
-    <row r="6" spans="1:12">
+    <row r="6" spans="8:8">
       <c r="H6" s="4"/>
     </row>
-    <row r="8" spans="1:12">
+    <row r="8" spans="8:11">
       <c r="H8" s="4"/>
       <c r="K8" s="4"/>
     </row>
-    <row r="9" spans="1:12">
+    <row r="9" spans="8:11">
       <c r="H9" s="4"/>
       <c r="K9" s="4"/>
     </row>
-    <row r="10" spans="1:12">
+    <row r="10" spans="8:11">
       <c r="H10" s="4"/>
       <c r="K10" s="4"/>
     </row>
-    <row r="11" spans="1:12">
+    <row r="11" spans="8:11">
       <c r="H11" s="4"/>
       <c r="K11" s="4"/>
     </row>
-    <row r="12" spans="1:12">
+    <row r="12" spans="8:11">
       <c r="H12" s="4"/>
       <c r="K12" s="4"/>
     </row>
-    <row r="13" spans="1:12">
+    <row r="13" spans="8:11">
       <c r="H13" s="4"/>
       <c r="K13" s="4"/>
     </row>
-    <row r="14" spans="1:12">
+    <row r="14" spans="8:11">
       <c r="H14" s="4"/>
       <c r="K14" s="4"/>
     </row>
-    <row r="15" spans="1:12">
+    <row r="15" spans="8:11">
       <c r="H15" s="4"/>
       <c r="K15" s="4"/>
     </row>
-    <row r="16" spans="1:12">
+    <row r="16" spans="8:11">
       <c r="H16" s="4"/>
       <c r="K16" s="4"/>
     </row>
@@ -2191,7 +2213,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:L13"/>
-  <sheetFormatPr defaultColWidth="9.14166666666667" defaultRowHeight="14"/>
+  <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="16.8"/>
   <sheetData>
     <row r="1" spans="1:12">
       <c r="A1" s="1" t="s">
@@ -2215,13 +2237,13 @@
       <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="H1" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="2"/>
-      <c r="J1" s="2"/>
-      <c r="K1" s="2"/>
-      <c r="L1" s="2"/>
+      <c r="I1" s="3"/>
+      <c r="J1" s="3"/>
+      <c r="K1" s="3"/>
+      <c r="L1" s="3"/>
     </row>
     <row r="2" spans="1:12">
       <c r="A2" s="1" t="s">
@@ -2249,14 +2271,14 @@
         <v>6</v>
       </c>
     </row>
-    <row r="3" ht="168" spans="1:12">
+    <row r="3" ht="219" spans="1:12">
       <c r="A3" s="1" t="s">
         <v>11</v>
       </c>
       <c r="B3" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="C3" s="2" t="s">
         <v>13</v>
       </c>
       <c r="D3" s="1" t="s">
@@ -2279,7 +2301,7 @@
       </c>
       <c r="L3" s="1"/>
     </row>
-    <row r="4" spans="1:12">
+    <row r="4" spans="2:10">
       <c r="B4" t="s">
         <v>69</v>
       </c>
@@ -2293,49 +2315,189 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:12">
+    <row r="5" spans="8:8">
       <c r="H5" s="4" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="6" spans="1:12">
+    <row r="6" spans="8:8">
       <c r="H6" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="7" spans="1:12">
+    <row r="7" spans="8:8">
       <c r="H7" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="8" spans="1:12">
+    <row r="8" spans="8:8">
       <c r="H8" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="9" spans="1:12">
+    <row r="9" spans="8:8">
       <c r="H9" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="10" spans="1:12">
+    <row r="10" spans="8:8">
       <c r="H10" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="11" spans="1:12">
+    <row r="11" spans="8:8">
       <c r="H11" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="12" spans="1:12">
+    <row r="12" spans="8:8">
       <c r="H12" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="13" spans="1:12">
+    <row r="13" spans="8:8">
       <c r="H13" t="s">
         <v>79</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="H1:L1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="A1:L9"/>
+  <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="16.8"/>
+  <sheetData>
+    <row r="1" spans="1:12">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="3"/>
+      <c r="J1" s="3"/>
+      <c r="K1" s="3"/>
+      <c r="L1" s="3"/>
+    </row>
+    <row r="2" spans="1:12">
+      <c r="A2" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="1"/>
+      <c r="C2" s="1"/>
+      <c r="D2" s="1"/>
+      <c r="E2" s="1"/>
+      <c r="F2" s="1"/>
+      <c r="G2" s="1"/>
+      <c r="H2" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="I2" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="J2" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="K2" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="L2" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="3" ht="219" spans="1:12">
+      <c r="A3" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="E3" s="1"/>
+      <c r="F3" s="1"/>
+      <c r="G3" s="1"/>
+      <c r="H3" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="I3" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="J3" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="K3" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="L3" s="1"/>
+    </row>
+    <row r="4" spans="2:10">
+      <c r="B4" t="s">
+        <v>80</v>
+      </c>
+      <c r="D4" t="b">
+        <v>1</v>
+      </c>
+      <c r="H4" t="s">
+        <v>81</v>
+      </c>
+      <c r="J4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="8:8">
+      <c r="H5" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="6" spans="8:8">
+      <c r="H6" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="7" spans="8:8">
+      <c r="H7" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="8" spans="8:8">
+      <c r="H8" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="9" spans="8:8">
+      <c r="H9" t="s">
+        <v>86</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add EndTurn card & auto-number generated effects
Change CardEffectGeneratorEditor to emit zero-padded numeric prefixes for generated card effect files, ensuring deterministic ordering. Add a new card entry (结束回合, id=34) to cardtable.json and CardEnum. Rename many existing card effect scripts to numbered filenames and add corresponding .meta files. Add a SpriteConfig asset and runtime SpriteConfig.cs. Update scenes and UI prefabs to wire maskText/Broader UI elements and adjust references (GamePlay.unity, 02UICardVisual.prefab), and apply related minor formatting and code cleanups across gameplay/UI scripts and config spreadsheets.
</commit_message>
<xml_diff>
--- a/Configs/source/Datas/__enums__.xlsx
+++ b/Configs/source/Datas/__enums__.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="29100" windowHeight="12700" firstSheet="2" activeTab="6"/>
+    <workbookView windowWidth="29100" windowHeight="12700" firstSheet="2"/>
   </bookViews>
   <sheets>
     <sheet name="Card" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="223" uniqueCount="87">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="224" uniqueCount="88">
   <si>
     <t>##var</t>
   </si>
@@ -195,6 +195,9 @@
   </si>
   <si>
     <t>二郎神请神</t>
+  </si>
+  <si>
+    <t>结束回合</t>
   </si>
   <si>
     <t>CardTypeEnum</t>
@@ -1300,7 +1303,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:L37"/>
+  <dimension ref="A1:L38"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="16.8"/>
   <cols>
     <col min="2" max="2" width="19" customWidth="1"/>
@@ -1574,6 +1577,11 @@
     <row r="37" spans="8:8">
       <c r="H37" s="6" t="s">
         <v>53</v>
+      </c>
+    </row>
+    <row r="38" spans="8:8">
+      <c r="H38" t="s">
+        <v>54</v>
       </c>
     </row>
   </sheetData>
@@ -1691,28 +1699,28 @@
     </row>
     <row r="4" customFormat="1" spans="2:8">
       <c r="B4" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="D4" t="b">
         <v>1</v>
       </c>
       <c r="H4" s="5" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="5" customFormat="1" spans="8:8">
       <c r="H5" s="5" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="6" customFormat="1" spans="8:8">
       <c r="H6" s="5" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
     </row>
     <row r="7" customFormat="1" spans="8:8">
       <c r="H7" s="5" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="8" customFormat="1" spans="8:8">
@@ -1863,18 +1871,18 @@
     </row>
     <row r="4" spans="2:8">
       <c r="B4" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="D4" t="b">
         <v>1</v>
       </c>
       <c r="H4" s="4" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
     </row>
     <row r="5" spans="8:8">
       <c r="H5" s="4" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
     </row>
     <row r="6" spans="8:8">
@@ -1986,28 +1994,28 @@
     </row>
     <row r="4" spans="2:8">
       <c r="B4" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D4" t="b">
         <v>1</v>
       </c>
       <c r="H4" s="4" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="5" spans="8:8">
       <c r="H5" s="4" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
     </row>
     <row r="6" spans="8:8">
       <c r="H6" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
     </row>
     <row r="7" spans="8:8">
       <c r="H7" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
   </sheetData>
@@ -2118,19 +2126,19 @@
     </row>
     <row r="4" spans="2:11">
       <c r="B4" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="D4" t="b">
         <v>1</v>
       </c>
       <c r="H4" s="4" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="J4">
         <v>-1</v>
       </c>
       <c r="K4" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
     </row>
     <row r="6" spans="8:8">
@@ -2303,13 +2311,13 @@
     </row>
     <row r="4" spans="2:10">
       <c r="B4" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="D4" t="b">
         <v>1</v>
       </c>
       <c r="H4" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="J4">
         <v>0</v>
@@ -2317,47 +2325,47 @@
     </row>
     <row r="5" spans="8:8">
       <c r="H5" s="4" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
     </row>
     <row r="6" spans="8:8">
       <c r="H6" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
     </row>
     <row r="7" spans="8:8">
       <c r="H7" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
     </row>
     <row r="8" spans="8:8">
       <c r="H8" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="9" spans="8:8">
       <c r="H9" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
     </row>
     <row r="10" spans="8:8">
       <c r="H10" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
     </row>
     <row r="11" spans="8:8">
       <c r="H11" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
     </row>
     <row r="12" spans="8:8">
       <c r="H12" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="13" spans="8:8">
       <c r="H13" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
     </row>
   </sheetData>
@@ -2463,13 +2471,13 @@
     </row>
     <row r="4" spans="2:10">
       <c r="B4" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="D4" t="b">
         <v>1</v>
       </c>
       <c r="H4" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="J4">
         <v>0</v>
@@ -2477,27 +2485,27 @@
     </row>
     <row r="5" spans="8:8">
       <c r="H5" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
     </row>
     <row r="6" spans="8:8">
       <c r="H6" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
     </row>
     <row r="7" spans="8:8">
       <c r="H7" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
     </row>
     <row r="8" spans="8:8">
       <c r="H8" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
     </row>
     <row r="9" spans="8:8">
       <c r="H9" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
     </row>
   </sheetData>

</xml_diff>